<commit_message>
Updates to OMS mapping
</commit_message>
<xml_diff>
--- a/ssn/rdf/ontology/alignments/sosa-mappings-sssom.xlsx
+++ b/ssn/rdf/ontology/alignments/sosa-mappings-sssom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\W3C\sdw-sosa-ssn\ssn\mappings\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\W3C\sdw-sosa-ssn\ssn\rdf\ontology\alignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{229D45CE-5274-4CE0-9DAB-98EE326EBBEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3160E948-8609-467D-8AB5-02650959F8F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14310" yWindow="2745" windowWidth="21270" windowHeight="14295" xr2:uid="{00E2F0C7-36F4-48CD-AB7C-87DDD7B41E94}"/>
+    <workbookView xWindow="17925" yWindow="1095" windowWidth="20505" windowHeight="19680" activeTab="1" xr2:uid="{00E2F0C7-36F4-48CD-AB7C-87DDD7B41E94}"/>
   </bookViews>
   <sheets>
     <sheet name="SSN-SDO" sheetId="11" r:id="rId1"/>
@@ -574,7 +574,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="408">
   <si>
     <t>subject_id</t>
   </si>
@@ -1579,9 +1579,6 @@
     <t>sam-cpt:Sampling/sample-sem</t>
   </si>
   <si>
-    <t>sosa:hasSampledFeature</t>
-  </si>
-  <si>
     <t>sam-cpt:Sample/sampledFeature-sem</t>
   </si>
   <si>
@@ -1790,6 +1787,18 @@
   </si>
   <si>
     <t>schema:startTime</t>
+  </si>
+  <si>
+    <t>obs-basic:ObservationCollection</t>
+  </si>
+  <si>
+    <t>sosa:isSampleOfUltimateFOI</t>
+  </si>
+  <si>
+    <t>sosa:usedForExecution</t>
+  </si>
+  <si>
+    <t>sosa:wasObservedBy</t>
   </si>
 </sst>
 </file>
@@ -1938,19 +1947,19 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -2624,7 +2633,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B2" t="s">
         <v>225</v>
@@ -2644,7 +2653,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B3" t="s">
         <v>225</v>
@@ -2664,13 +2673,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B4" t="s">
         <v>206</v>
       </c>
       <c r="C4" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -2690,7 +2699,7 @@
         <v>206</v>
       </c>
       <c r="C5" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -2704,13 +2713,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B6" t="s">
         <v>206</v>
       </c>
       <c r="C6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -2730,7 +2739,7 @@
         <v>206</v>
       </c>
       <c r="C7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
@@ -2750,7 +2759,7 @@
         <v>206</v>
       </c>
       <c r="C8" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -2770,7 +2779,7 @@
         <v>206</v>
       </c>
       <c r="C9" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -2790,7 +2799,7 @@
         <v>206</v>
       </c>
       <c r="C10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -2804,13 +2813,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B11" t="s">
         <v>206</v>
       </c>
       <c r="C11" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
@@ -2824,13 +2833,13 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B12" t="s">
         <v>206</v>
       </c>
       <c r="C12" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
@@ -2844,13 +2853,13 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B13" t="s">
         <v>206</v>
       </c>
       <c r="C13" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D13" t="s">
         <v>10</v>
@@ -2864,13 +2873,13 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B14" t="s">
         <v>206</v>
       </c>
       <c r="C14" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D14" t="s">
         <v>10</v>
@@ -2890,7 +2899,7 @@
         <v>206</v>
       </c>
       <c r="C15" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
@@ -2910,7 +2919,7 @@
         <v>206</v>
       </c>
       <c r="C16" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
@@ -2930,7 +2939,7 @@
         <v>206</v>
       </c>
       <c r="C17" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D17" t="s">
         <v>10</v>
@@ -2950,7 +2959,7 @@
         <v>206</v>
       </c>
       <c r="C18" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
@@ -2970,7 +2979,7 @@
         <v>206</v>
       </c>
       <c r="C19" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
@@ -2990,7 +2999,7 @@
         <v>206</v>
       </c>
       <c r="C20" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
@@ -3010,7 +3019,7 @@
         <v>206</v>
       </c>
       <c r="C21" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
@@ -3030,7 +3039,7 @@
         <v>225</v>
       </c>
       <c r="C22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
@@ -3050,7 +3059,7 @@
         <v>225</v>
       </c>
       <c r="C23" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
@@ -3070,7 +3079,7 @@
         <v>225</v>
       </c>
       <c r="C24" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
@@ -3090,7 +3099,7 @@
         <v>225</v>
       </c>
       <c r="C25" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
@@ -3110,7 +3119,7 @@
         <v>225</v>
       </c>
       <c r="C26" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -3130,7 +3139,7 @@
         <v>225</v>
       </c>
       <c r="C27" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
@@ -3150,7 +3159,7 @@
         <v>225</v>
       </c>
       <c r="C28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
@@ -3170,7 +3179,7 @@
         <v>225</v>
       </c>
       <c r="C29" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -3190,7 +3199,7 @@
         <v>225</v>
       </c>
       <c r="C30" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -3210,7 +3219,7 @@
         <v>225</v>
       </c>
       <c r="C31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -3251,7 +3260,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B5BDD32-D80B-4775-8CB1-BF5BF87D513D}">
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" customWidth="1"/>
@@ -3316,7 +3325,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B3" t="s">
         <v>306</v>
@@ -3336,7 +3345,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="B4" t="s">
         <v>306</v>
@@ -3376,13 +3385,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>374</v>
+        <v>207</v>
       </c>
       <c r="B6" t="s">
         <v>306</v>
       </c>
       <c r="C6" t="s">
-        <v>311</v>
+        <v>404</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -3396,13 +3405,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>253</v>
+        <v>373</v>
       </c>
       <c r="B7" t="s">
         <v>306</v>
       </c>
       <c r="C7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
@@ -3416,13 +3425,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>375</v>
+        <v>253</v>
       </c>
       <c r="B8" t="s">
         <v>306</v>
       </c>
       <c r="C8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -3436,13 +3445,13 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>314</v>
+        <v>374</v>
       </c>
       <c r="B9" t="s">
         <v>306</v>
       </c>
       <c r="C9" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -3456,13 +3465,13 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>216</v>
+        <v>314</v>
       </c>
       <c r="B10" t="s">
         <v>306</v>
       </c>
       <c r="C10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -3476,13 +3485,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>278</v>
+        <v>216</v>
       </c>
       <c r="B11" t="s">
         <v>306</v>
       </c>
       <c r="C11" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
@@ -3496,13 +3505,13 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>318</v>
+        <v>278</v>
       </c>
       <c r="B12" t="s">
         <v>306</v>
       </c>
       <c r="C12" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
@@ -3516,13 +3525,13 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>277</v>
+        <v>318</v>
       </c>
       <c r="B13" t="s">
         <v>306</v>
       </c>
       <c r="C13" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D13" t="s">
         <v>10</v>
@@ -3536,13 +3545,13 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B14" t="s">
         <v>306</v>
       </c>
       <c r="C14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D14" t="s">
         <v>10</v>
@@ -3556,13 +3565,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>376</v>
+        <v>274</v>
       </c>
       <c r="B15" t="s">
         <v>306</v>
       </c>
       <c r="C15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
@@ -3576,13 +3585,13 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>249</v>
+        <v>375</v>
       </c>
       <c r="B16" t="s">
         <v>306</v>
       </c>
       <c r="C16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
@@ -3596,13 +3605,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>377</v>
+        <v>249</v>
       </c>
       <c r="B17" t="s">
         <v>306</v>
       </c>
       <c r="C17" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D17" t="s">
         <v>10</v>
@@ -3616,13 +3625,13 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B18" t="s">
         <v>306</v>
       </c>
       <c r="C18" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
@@ -3636,13 +3645,13 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>267</v>
+        <v>377</v>
       </c>
       <c r="B19" t="s">
         <v>306</v>
       </c>
       <c r="C19" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
@@ -3656,13 +3665,13 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B20" t="s">
         <v>306</v>
       </c>
       <c r="C20" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
@@ -3676,13 +3685,13 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B21" t="s">
         <v>306</v>
       </c>
       <c r="C21" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
@@ -3696,13 +3705,13 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>226</v>
+        <v>268</v>
       </c>
       <c r="B22" t="s">
         <v>306</v>
       </c>
       <c r="C22" t="s">
-        <v>379</v>
+        <v>328</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
@@ -3722,7 +3731,7 @@
         <v>306</v>
       </c>
       <c r="C23" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
@@ -3742,7 +3751,7 @@
         <v>306</v>
       </c>
       <c r="C24" t="s">
-        <v>329</v>
+        <v>379</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
@@ -3756,13 +3765,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B25" t="s">
         <v>306</v>
       </c>
       <c r="C25" t="s">
-        <v>381</v>
+        <v>329</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
@@ -3782,7 +3791,7 @@
         <v>306</v>
       </c>
       <c r="C26" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -3796,13 +3805,13 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>331</v>
+        <v>232</v>
       </c>
       <c r="B27" t="s">
         <v>306</v>
       </c>
       <c r="C27" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
@@ -3816,13 +3825,13 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>229</v>
+        <v>331</v>
       </c>
       <c r="B28" t="s">
         <v>306</v>
       </c>
       <c r="C28" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
@@ -3842,7 +3851,7 @@
         <v>306</v>
       </c>
       <c r="C29" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -3856,13 +3865,13 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>334</v>
+        <v>229</v>
       </c>
       <c r="B30" t="s">
         <v>306</v>
       </c>
       <c r="C30" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -3876,13 +3885,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B31" t="s">
         <v>306</v>
       </c>
       <c r="C31" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -3896,13 +3905,13 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B32" t="s">
         <v>306</v>
       </c>
       <c r="C32" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D32" t="s">
         <v>10</v>
@@ -3922,7 +3931,7 @@
         <v>306</v>
       </c>
       <c r="C33" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -3942,7 +3951,7 @@
         <v>306</v>
       </c>
       <c r="C34" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
@@ -3962,7 +3971,7 @@
         <v>306</v>
       </c>
       <c r="C35" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
@@ -3982,7 +3991,7 @@
         <v>306</v>
       </c>
       <c r="C36" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
@@ -4002,7 +4011,7 @@
         <v>306</v>
       </c>
       <c r="C37" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
@@ -4022,7 +4031,7 @@
         <v>306</v>
       </c>
       <c r="C38" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D38" t="s">
         <v>10</v>
@@ -4036,13 +4045,13 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B39" t="s">
         <v>306</v>
       </c>
       <c r="C39" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -4056,13 +4065,13 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B40" t="s">
         <v>306</v>
       </c>
       <c r="C40" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
@@ -4082,7 +4091,7 @@
         <v>306</v>
       </c>
       <c r="C41" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D41" t="s">
         <v>10</v>
@@ -4096,13 +4105,13 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>280</v>
+        <v>405</v>
       </c>
       <c r="B42" t="s">
         <v>306</v>
       </c>
       <c r="C42" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="D42" t="s">
         <v>10</v>
@@ -4116,13 +4125,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
       <c r="B43" t="s">
         <v>306</v>
       </c>
       <c r="C43" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D43" t="s">
         <v>10</v>
@@ -4136,13 +4145,13 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B44" t="s">
         <v>306</v>
       </c>
       <c r="C44" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D44" t="s">
         <v>10</v>
@@ -4156,13 +4165,13 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>349</v>
+        <v>261</v>
       </c>
       <c r="B45" t="s">
         <v>306</v>
       </c>
       <c r="C45" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="D45" t="s">
         <v>10</v>
@@ -4176,13 +4185,13 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B46" t="s">
         <v>306</v>
       </c>
       <c r="C46" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="D46" t="s">
         <v>10</v>
@@ -4196,13 +4205,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B47" t="s">
         <v>306</v>
       </c>
       <c r="C47" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -4216,13 +4225,13 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B48" t="s">
         <v>306</v>
       </c>
       <c r="C48" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -4236,13 +4245,13 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>227</v>
+        <v>354</v>
       </c>
       <c r="B49" t="s">
         <v>306</v>
       </c>
       <c r="C49" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D49" t="s">
         <v>10</v>
@@ -4256,13 +4265,13 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>358</v>
+        <v>227</v>
       </c>
       <c r="B50" t="s">
         <v>306</v>
       </c>
       <c r="C50" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D50" t="s">
         <v>10</v>
@@ -4276,13 +4285,13 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>264</v>
+        <v>357</v>
       </c>
       <c r="B51" t="s">
         <v>306</v>
       </c>
       <c r="C51" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D51" t="s">
         <v>10</v>
@@ -4296,13 +4305,13 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>361</v>
+        <v>264</v>
       </c>
       <c r="B52" t="s">
         <v>306</v>
       </c>
       <c r="C52" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D52" t="s">
         <v>10</v>
@@ -4316,13 +4325,13 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B53" t="s">
         <v>306</v>
       </c>
       <c r="C53" t="s">
-        <v>341</v>
+        <v>361</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
@@ -4336,13 +4345,13 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>385</v>
+        <v>362</v>
       </c>
       <c r="B54" t="s">
         <v>306</v>
       </c>
       <c r="C54" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -4356,13 +4365,13 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>364</v>
+        <v>384</v>
       </c>
       <c r="B55" t="s">
         <v>306</v>
       </c>
       <c r="C55" t="s">
-        <v>365</v>
+        <v>343</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
@@ -4376,13 +4385,13 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="B56" t="s">
         <v>306</v>
       </c>
       <c r="C56" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D56" t="s">
         <v>10</v>
@@ -4396,13 +4405,13 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>284</v>
+        <v>385</v>
       </c>
       <c r="B57" t="s">
         <v>306</v>
       </c>
       <c r="C57" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D57" t="s">
         <v>10</v>
@@ -4416,13 +4425,13 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>368</v>
+        <v>284</v>
       </c>
       <c r="B58" t="s">
         <v>306</v>
       </c>
       <c r="C58" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="D58" t="s">
         <v>10</v>
@@ -4436,13 +4445,13 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>228</v>
+        <v>367</v>
       </c>
       <c r="B59" t="s">
         <v>306</v>
       </c>
       <c r="C59" t="s">
-        <v>384</v>
+        <v>368</v>
       </c>
       <c r="D59" t="s">
         <v>10</v>
@@ -4456,13 +4465,13 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>228</v>
+        <v>406</v>
       </c>
       <c r="B60" t="s">
         <v>306</v>
       </c>
       <c r="C60" t="s">
-        <v>370</v>
+        <v>343</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
@@ -4476,13 +4485,13 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>371</v>
+        <v>228</v>
       </c>
       <c r="B61" t="s">
         <v>306</v>
       </c>
       <c r="C61" t="s">
-        <v>372</v>
+        <v>383</v>
       </c>
       <c r="D61" t="s">
         <v>10</v>
@@ -4491,12 +4500,72 @@
         <v>234</v>
       </c>
       <c r="F61">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>228</v>
+      </c>
+      <c r="B62" t="s">
+        <v>306</v>
+      </c>
+      <c r="C62" t="s">
+        <v>369</v>
+      </c>
+      <c r="D62" t="s">
+        <v>10</v>
+      </c>
+      <c r="E62" t="s">
+        <v>234</v>
+      </c>
+      <c r="F62">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>370</v>
+      </c>
+      <c r="B63" t="s">
+        <v>306</v>
+      </c>
+      <c r="C63" t="s">
+        <v>371</v>
+      </c>
+      <c r="D63" t="s">
+        <v>10</v>
+      </c>
+      <c r="E63" t="s">
+        <v>234</v>
+      </c>
+      <c r="F63">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>407</v>
+      </c>
+      <c r="B64" t="s">
+        <v>306</v>
+      </c>
+      <c r="C64" t="s">
+        <v>343</v>
+      </c>
+      <c r="D64" t="s">
+        <v>10</v>
+      </c>
+      <c r="E64" t="s">
+        <v>234</v>
+      </c>
+      <c r="F64">
         <v>2024</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation errorStyle="warning" showInputMessage="1" showErrorMessage="1" promptTitle="predicates" prompt="Select mapping predicate" sqref="A8:A12 C8:C12 B1:B1048576" xr:uid="{E137DD0E-8745-4BDC-9B77-0C448A1AFF20}"/>
+    <dataValidation errorStyle="warning" showInputMessage="1" showErrorMessage="1" promptTitle="predicates" prompt="Select mapping predicate" sqref="A9:A13 C9:C13 B1:B1048576" xr:uid="{E137DD0E-8745-4BDC-9B77-0C448A1AFF20}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -4580,7 +4649,7 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F2">
         <v>2017</v>
@@ -4600,7 +4669,7 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F3">
         <v>2017</v>
@@ -4620,7 +4689,7 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F4">
         <v>2017</v>
@@ -4640,7 +4709,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F5">
         <v>2017</v>
@@ -4660,7 +4729,7 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F6">
         <v>2017</v>
@@ -4680,7 +4749,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F7">
         <v>2017</v>
@@ -4700,7 +4769,7 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F8">
         <v>2017</v>
@@ -4720,7 +4789,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F9">
         <v>2017</v>
@@ -4740,7 +4809,7 @@
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F10">
         <v>2017</v>
@@ -4760,7 +4829,7 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F11">
         <v>2017</v>
@@ -4780,7 +4849,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F12">
         <v>2017</v>
@@ -4800,7 +4869,7 @@
         <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F13">
         <v>2017</v>
@@ -4820,7 +4889,7 @@
         <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F14">
         <v>2017</v>
@@ -4840,7 +4909,7 @@
         <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F15">
         <v>2017</v>
@@ -4860,7 +4929,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F16">
         <v>2017</v>
@@ -4880,7 +4949,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F17">
         <v>2017</v>
@@ -4900,7 +4969,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F18">
         <v>2017</v>
@@ -4920,7 +4989,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F19">
         <v>2017</v>
@@ -4940,7 +5009,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F20">
         <v>2017</v>
@@ -4960,7 +5029,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F21">
         <v>2017</v>
@@ -4980,7 +5049,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F22">
         <v>2017</v>
@@ -5000,7 +5069,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F23">
         <v>2017</v>
@@ -5020,7 +5089,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F24">
         <v>2017</v>
@@ -5034,7 +5103,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F25">
         <v>2017</v>
@@ -5126,7 +5195,7 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F2">
         <v>2017</v>
@@ -5146,7 +5215,7 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F3">
         <v>2017</v>
@@ -5166,7 +5235,7 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F4">
         <v>2017</v>
@@ -5186,7 +5255,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F5">
         <v>2017</v>
@@ -5206,7 +5275,7 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F6">
         <v>2017</v>
@@ -5226,7 +5295,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F7">
         <v>2017</v>
@@ -5246,7 +5315,7 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F8">
         <v>2017</v>
@@ -5266,7 +5335,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F9">
         <v>2017</v>
@@ -5286,7 +5355,7 @@
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F10">
         <v>2017</v>
@@ -5306,7 +5375,7 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F11">
         <v>2017</v>
@@ -5326,7 +5395,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F12">
         <v>2017</v>
@@ -5346,7 +5415,7 @@
         <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F13">
         <v>2017</v>
@@ -5366,7 +5435,7 @@
         <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F14">
         <v>2017</v>
@@ -5386,7 +5455,7 @@
         <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F15">
         <v>2017</v>
@@ -5406,7 +5475,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F16">
         <v>2017</v>
@@ -5426,7 +5495,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F17">
         <v>2017</v>
@@ -5446,7 +5515,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F18">
         <v>2017</v>
@@ -5466,7 +5535,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F19">
         <v>2017</v>
@@ -5486,7 +5555,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F20">
         <v>2017</v>
@@ -5506,7 +5575,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F21">
         <v>2017</v>
@@ -5526,7 +5595,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F22">
         <v>2017</v>
@@ -5546,7 +5615,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F23">
         <v>2017</v>
@@ -5566,7 +5635,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F24">
         <v>2017</v>
@@ -5586,7 +5655,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F25">
         <v>2017</v>
@@ -5606,7 +5675,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F26">
         <v>2017</v>
@@ -5626,7 +5695,7 @@
         <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F27">
         <v>2017</v>
@@ -6227,7 +6296,7 @@
     </row>
     <row r="6" spans="1:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="4"/>
@@ -6368,27 +6437,27 @@
     </row>
     <row r="24" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="G24" s="9"/>
-      <c r="H24" s="11"/>
+      <c r="H24" s="12"/>
       <c r="I24" s="6"/>
     </row>
     <row r="25" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="G25" s="13"/>
-      <c r="H25" s="14"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="13"/>
       <c r="I25" s="7"/>
     </row>
     <row r="26" spans="1:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G26" s="10"/>
-      <c r="H26" s="12"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="14"/>
       <c r="I26" s="8"/>
     </row>
     <row r="27" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="G27" s="9"/>
-      <c r="H27" s="11"/>
+      <c r="H27" s="12"/>
       <c r="I27" s="6"/>
     </row>
     <row r="28" spans="1:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G28" s="10"/>
-      <c r="H28" s="12"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="14"/>
       <c r="I28" s="8"/>
     </row>
     <row r="29" spans="1:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6398,12 +6467,12 @@
     </row>
     <row r="30" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="G30" s="9"/>
-      <c r="H30" s="11"/>
+      <c r="H30" s="12"/>
       <c r="I30" s="6"/>
     </row>
     <row r="31" spans="1:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G31" s="10"/>
-      <c r="H31" s="12"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="14"/>
       <c r="I31" s="8"/>
     </row>
     <row r="32" spans="1:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6423,27 +6492,27 @@
     </row>
     <row r="35" spans="7:9" ht="18" x14ac:dyDescent="0.25">
       <c r="G35" s="9"/>
-      <c r="H35" s="11"/>
+      <c r="H35" s="12"/>
       <c r="I35" s="6"/>
     </row>
     <row r="36" spans="7:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G36" s="10"/>
-      <c r="H36" s="12"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="14"/>
       <c r="I36" s="8"/>
     </row>
     <row r="37" spans="7:9" ht="18" x14ac:dyDescent="0.25">
       <c r="G37" s="9"/>
-      <c r="H37" s="11"/>
+      <c r="H37" s="12"/>
       <c r="I37" s="6"/>
     </row>
     <row r="38" spans="7:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="G38" s="13"/>
-      <c r="H38" s="14"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="13"/>
       <c r="I38" s="7"/>
     </row>
     <row r="39" spans="7:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G39" s="10"/>
-      <c r="H39" s="12"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="14"/>
       <c r="I39" s="8"/>
     </row>
     <row r="40" spans="7:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6553,12 +6622,12 @@
     </row>
     <row r="61" spans="7:9" ht="18" x14ac:dyDescent="0.25">
       <c r="G61" s="9"/>
-      <c r="H61" s="11"/>
+      <c r="H61" s="12"/>
       <c r="I61" s="6"/>
     </row>
     <row r="62" spans="7:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G62" s="10"/>
-      <c r="H62" s="12"/>
+      <c r="G62" s="11"/>
+      <c r="H62" s="14"/>
       <c r="I62" s="8"/>
     </row>
     <row r="63" spans="7:9" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6568,18 +6637,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="G37:G39"/>
+    <mergeCell ref="H37:H39"/>
+    <mergeCell ref="G61:G62"/>
+    <mergeCell ref="H61:H62"/>
     <mergeCell ref="G24:G26"/>
     <mergeCell ref="H24:H26"/>
     <mergeCell ref="G27:G28"/>
     <mergeCell ref="H27:H28"/>
     <mergeCell ref="G30:G31"/>
     <mergeCell ref="H30:H31"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="G37:G39"/>
-    <mergeCell ref="H37:H39"/>
-    <mergeCell ref="G61:G62"/>
-    <mergeCell ref="H61:H62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>